<commit_message>
Load public SOOP profile images by ID independent of LIVE status
</commit_message>
<xml_diff>
--- a/downloads/wapobook-admin-template.xlsx
+++ b/downloads/wapobook-admin-template.xlsx
@@ -805,7 +805,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>사진 열은 없습니다. 승인된 SOOP 조회 결과를 계정ID로 연결합니다. 기존 사진은 덮어쓰지 않습니다.</t>
+          <t>사진 열은 없습니다. 관리자에서 ID로 프로필 사진 조회를 눌러 원본 이미지 로드를 확인하고 승인합니다. 기존 사진은 덮어쓰지 않습니다.</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>요청 JSON 다운로드 → 검수된 공급자 설정 → GitHub Actions 수동 실행 → 결과 JSON 업로드 → 사진 미리보기 승인. 토큰은 엑셀이나 브라우저에 넣지 마세요.</t>
+          <t>엑셀 업로드 → ID로 프로필 사진 조회 → 이미지 미리보기 확인 → 병합 승인. 방송 여부는 조회하지 않습니다. 실패하면 수동 사진 등록을 사용하세요.</t>
         </is>
       </c>
     </row>

</xml_diff>